<commit_message>
feat: update Excel credit risk prototype
</commit_message>
<xml_diff>
--- a/reports/excel/synthetic_credit_risk_prototype.xlsx
+++ b/reports/excel/synthetic_credit_risk_prototype.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\credit-risk-decision-system\reports\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B4B0A19B-4C68-4C8E-B8AF-EAE767590C0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC7D1F34-FFCA-43B5-8A96-A804670B38BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{BBB7CC6D-377D-4AE4-9941-B0252BEF4F25}"/>
+    <workbookView xWindow="1550" yWindow="1520" windowWidth="23040" windowHeight="13400" xr2:uid="{BBB7CC6D-377D-4AE4-9941-B0252BEF4F25}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>Applicant_ID</t>
   </si>
@@ -99,15 +99,23 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Application Lookup</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>A006</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
     <t>Credit Score</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Risk Threshold</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>High-Risk Defaults</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Applicant Lookup</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -116,9 +124,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="178" formatCode="[$$-1009]#,##0_);[Red]\([$$-1009]#,##0\)"/>
-    <numFmt numFmtId="179" formatCode="0.0%"/>
-    <numFmt numFmtId="180" formatCode="_-[$$-1009]* #,##0.00_-;\-[$$-1009]* #,##0.00_-;_-[$$-1009]* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="176" formatCode="[$$-1009]#,##0_);[Red]\([$$-1009]#,##0\)"/>
+    <numFmt numFmtId="177" formatCode="0.0%"/>
+    <numFmt numFmtId="178" formatCode="_-[$$-1009]* #,##0.00_-;\-[$$-1009]* #,##0.00_-;_-[$$-1009]* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -174,13 +182,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -188,7 +196,10 @@
     <cellStyle name="百分比" xfId="1" builtinId="5"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="7">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -217,40 +228,13 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
+      <numFmt numFmtId="177" formatCode="0.0%"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
+      <numFmt numFmtId="176" formatCode="[$$-1009]#,##0_);[Red]\([$$-1009]#,##0\)"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="179" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="178" formatCode="[$$-1009]#,##0_);[Red]\([$$-1009]#,##0\)"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="178" formatCode="[$$-1009]#,##0_);[Red]\([$$-1009]#,##0\)"/>
+      <numFmt numFmtId="176" formatCode="[$$-1009]#,##0_);[Red]\([$$-1009]#,##0\)"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -300,7 +284,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US" altLang="zh-CN"/>
-              <a:t>Debt_to_Income by Application</a:t>
+              <a:t>Debt_to_Income by Applicant</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -1247,15 +1231,15 @@
   </sortState>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{5DB3054D-B453-4F4B-ABDE-676A06796AF5}" name="Applicant_ID"/>
-    <tableColumn id="2" xr3:uid="{C84C28F8-3796-47D7-9032-662F1557773A}" name="Income" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{9BFBAFA3-DE7A-4B0C-957A-D916E0E54EEB}" name="Debt" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{C84C28F8-3796-47D7-9032-662F1557773A}" name="Income" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{9BFBAFA3-DE7A-4B0C-957A-D916E0E54EEB}" name="Debt" dataDxfId="5"/>
     <tableColumn id="4" xr3:uid="{DC3D9AA5-71BF-43FA-9B0E-8A4F6512FB97}" name="Credit_Score"/>
     <tableColumn id="5" xr3:uid="{78414401-7D35-4508-9F47-09AEC9F83448}" name="Defaulted"/>
-    <tableColumn id="6" xr3:uid="{6C483C90-A97B-4157-8B4B-2DED3C5C25D4}" name="Debt_to_Income" dataDxfId="6" dataCellStyle="百分比">
+    <tableColumn id="6" xr3:uid="{6C483C90-A97B-4157-8B4B-2DED3C5C25D4}" name="Debt_to_Income" dataDxfId="4" dataCellStyle="百分比">
       <calculatedColumnFormula>表1[[#This Row],[Debt]]/表1[[#This Row],[Income]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{68BC03E3-32DD-4531-87E8-8A72C88C7D4F}" name="Risk_Flag" dataDxfId="7">
-      <calculatedColumnFormula>IF(表1[[#This Row],[Credit_Score]]&lt;650, "High", "Low")</calculatedColumnFormula>
+    <tableColumn id="7" xr3:uid="{68BC03E3-32DD-4531-87E8-8A72C88C7D4F}" name="Risk_Flag" dataDxfId="0">
+      <calculatedColumnFormula>IF(表1[[#This Row],[Credit_Score]]&lt; $J$9, "High", "Low")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1579,7 +1563,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE3DCBB2-C9DD-4A72-8874-F973E3C8B88B}">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.08203125" customWidth="1"/>
@@ -1642,7 +1626,7 @@
         <v>0.20833333333333334</v>
       </c>
       <c r="G2" t="str">
-        <f>IF(表1[[#This Row],[Credit_Score]]&lt;650, "High", "Low")</f>
+        <f>IF(表1[[#This Row],[Credit_Score]]&lt; $J$9, "High", "Low")</f>
         <v>Low</v>
       </c>
       <c r="I2" t="s">
@@ -1674,7 +1658,7 @@
         <v>0.16666666666666666</v>
       </c>
       <c r="G3" t="str">
-        <f>IF(表1[[#This Row],[Credit_Score]]&lt;650, "High", "Low")</f>
+        <f>IF(表1[[#This Row],[Credit_Score]]&lt; $J$9, "High", "Low")</f>
         <v>Low</v>
       </c>
       <c r="I3" t="s">
@@ -1706,7 +1690,7 @@
         <v>0.25</v>
       </c>
       <c r="G4" t="str">
-        <f>IF(表1[[#This Row],[Credit_Score]]&lt;650, "High", "Low")</f>
+        <f>IF(表1[[#This Row],[Credit_Score]]&lt; $J$9, "High", "Low")</f>
         <v>Low</v>
       </c>
       <c r="I4" t="s">
@@ -1738,7 +1722,7 @@
         <v>0.5</v>
       </c>
       <c r="G5" t="str">
-        <f>IF(表1[[#This Row],[Credit_Score]]&lt;650, "High", "Low")</f>
+        <f>IF(表1[[#This Row],[Credit_Score]]&lt; $J$9, "High", "Low")</f>
         <v>High</v>
       </c>
     </row>
@@ -1763,14 +1747,14 @@
         <v>0.51428571428571423</v>
       </c>
       <c r="G6" t="str">
-        <f>IF(表1[[#This Row],[Credit_Score]]&lt;650, "High", "Low")</f>
+        <f>IF(表1[[#This Row],[Credit_Score]]&lt; $J$9, "High", "Low")</f>
         <v>High</v>
       </c>
       <c r="I6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J6" t="s">
         <v>18</v>
-      </c>
-      <c r="J6" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
@@ -1794,28 +1778,45 @@
         <v>0.53658536585365857</v>
       </c>
       <c r="G7" t="str">
-        <f>IF(表1[[#This Row],[Credit_Score]]&lt;650, "High", "Low")</f>
+        <f>IF(表1[[#This Row],[Credit_Score]]&lt; $J$9, "High", "Low")</f>
         <v>High</v>
       </c>
       <c r="I7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J7">
         <f>_xlfn.XLOOKUP(J6, 表1[Applicant_ID], 表1[Credit_Score], "Not Found")</f>
         <v>640</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I9" t="s">
+        <v>20</v>
+      </c>
+      <c r="J9">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I10" t="s">
+        <v>21</v>
+      </c>
+      <c r="J10">
+        <f>COUNTIFS(表1[Risk_Flag], "High", 表1[Defaulted], 1)</f>
+        <v>3</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="G2:G7">
-    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="High">
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Low">
+      <formula>NOT(ISERROR(SEARCH("Low",G2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="High">
       <formula>NOT(ISERROR(SEARCH("High",G2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="High">
+    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="High">
       <formula>NOT(ISERROR(SEARCH("High",G2)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Low">
-      <formula>NOT(ISERROR(SEARCH("Low",G2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
docs: update Excel prototype README
</commit_message>
<xml_diff>
--- a/reports/excel/synthetic_credit_risk_prototype.xlsx
+++ b/reports/excel/synthetic_credit_risk_prototype.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\credit-risk-decision-system\reports\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC7D1F34-FFCA-43B5-8A96-A804670B38BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5476D19E-1DB8-455B-A682-66E633D40C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1550" yWindow="1520" windowWidth="23040" windowHeight="13400" xr2:uid="{BBB7CC6D-377D-4AE4-9941-B0252BEF4F25}"/>
+    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{BBB7CC6D-377D-4AE4-9941-B0252BEF4F25}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>Applicant_ID</t>
   </si>
@@ -118,6 +118,30 @@
     <t>Applicant Lookup</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>Decision</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Decline Score Threshold</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Review DTI Threshold</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Approve</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Review</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Decline</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -178,7 +202,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -191,14 +215,64 @@
     <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="百分比" xfId="1" builtinId="5"/>
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="23">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <fill>
@@ -226,6 +300,103 @@
           <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="177" formatCode="0.0%"/>
@@ -639,7 +810,417 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="zh-CN"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" altLang="zh-CN"/>
+              <a:t>Decision Distribution</a:t>
+            </a:r>
+            <a:endParaRPr lang="zh-CN" altLang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.32915966754155729"/>
+          <c:y val="2.7777777777777776E-2"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="zh-CN"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="zh-CN"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$I$15:$I$17</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>Approve</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Review</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Decline</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$J$15:$J$17</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-503D-4FCB-90E5-5C05C2F24EE9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1799300640"/>
+        <c:axId val="1337053232"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1799300640"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="zh-CN"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1337053232"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1337053232"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="zh-CN"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1799300640"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="zh-CN"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -1182,20 +1763,523 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>927100</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>139700</xdr:rowOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>158750</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>107950</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>234950</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1263650</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>6350</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1220,26 +2304,65 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>273050</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>158750</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="图表 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{96D086E8-2EBC-7872-A330-C746F9527435}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{79CC04F0-4382-4F7E-97C9-60F422A61D94}" name="表1" displayName="表1" ref="A1:G7" totalsRowShown="0">
-  <autoFilter ref="A1:G7" xr:uid="{79CC04F0-4382-4F7E-97C9-60F422A61D94}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{79CC04F0-4382-4F7E-97C9-60F422A61D94}" name="表1" displayName="表1" ref="A1:H7" totalsRowShown="0">
+  <autoFilter ref="A1:H7" xr:uid="{79CC04F0-4382-4F7E-97C9-60F422A61D94}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:E7">
     <sortCondition descending="1" ref="D1:D7"/>
   </sortState>
-  <tableColumns count="7">
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{5DB3054D-B453-4F4B-ABDE-676A06796AF5}" name="Applicant_ID"/>
-    <tableColumn id="2" xr3:uid="{C84C28F8-3796-47D7-9032-662F1557773A}" name="Income" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{9BFBAFA3-DE7A-4B0C-957A-D916E0E54EEB}" name="Debt" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{C84C28F8-3796-47D7-9032-662F1557773A}" name="Income" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{9BFBAFA3-DE7A-4B0C-957A-D916E0E54EEB}" name="Debt" dataDxfId="21"/>
     <tableColumn id="4" xr3:uid="{DC3D9AA5-71BF-43FA-9B0E-8A4F6512FB97}" name="Credit_Score"/>
     <tableColumn id="5" xr3:uid="{78414401-7D35-4508-9F47-09AEC9F83448}" name="Defaulted"/>
-    <tableColumn id="6" xr3:uid="{6C483C90-A97B-4157-8B4B-2DED3C5C25D4}" name="Debt_to_Income" dataDxfId="4" dataCellStyle="百分比">
+    <tableColumn id="6" xr3:uid="{6C483C90-A97B-4157-8B4B-2DED3C5C25D4}" name="Debt_to_Income" dataDxfId="20" dataCellStyle="百分比">
       <calculatedColumnFormula>表1[[#This Row],[Debt]]/表1[[#This Row],[Income]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{68BC03E3-32DD-4531-87E8-8A72C88C7D4F}" name="Risk_Flag" dataDxfId="0">
+    <tableColumn id="7" xr3:uid="{68BC03E3-32DD-4531-87E8-8A72C88C7D4F}" name="Risk_Flag" dataDxfId="19">
       <calculatedColumnFormula>IF(表1[[#This Row],[Credit_Score]]&lt; $J$9, "High", "Low")</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="8" xr3:uid="{3075087F-CBFA-4972-B1FA-427EEF5F89D6}" name="Decision" dataDxfId="18">
+      <calculatedColumnFormula>IF(表1[[#This Row],[Credit_Score]]&lt;$J$12, "Decline", IF(表1[[#This Row],[Debt_to_Income]]&gt;=$J$13, "Review", "Approve"))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1563,16 +2686,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE3DCBB2-C9DD-4A72-8874-F973E3C8B88B}">
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.08203125" customWidth="1"/>
-    <col min="2" max="3" width="10.58203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="5" width="14.1640625" customWidth="1"/>
-    <col min="6" max="6" width="16.08203125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="18.25" customWidth="1"/>
-    <col min="9" max="9" width="20.25" customWidth="1"/>
+    <col min="1" max="1" width="13.9140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.08203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.83203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.75" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1598,6 +2723,9 @@
       <c r="G1" t="s">
         <v>12</v>
       </c>
+      <c r="H1" t="s">
+        <v>23</v>
+      </c>
       <c r="I1" t="s">
         <v>13</v>
       </c>
@@ -1629,6 +2757,10 @@
         <f>IF(表1[[#This Row],[Credit_Score]]&lt; $J$9, "High", "Low")</f>
         <v>Low</v>
       </c>
+      <c r="H2" t="str">
+        <f>IF(表1[[#This Row],[Credit_Score]]&lt;$J$12, "Decline", IF(表1[[#This Row],[Debt_to_Income]]&gt;=$J$13, "Review", "Approve"))</f>
+        <v>Approve</v>
+      </c>
       <c r="I2" t="s">
         <v>14</v>
       </c>
@@ -1661,6 +2793,10 @@
         <f>IF(表1[[#This Row],[Credit_Score]]&lt; $J$9, "High", "Low")</f>
         <v>Low</v>
       </c>
+      <c r="H3" t="str">
+        <f>IF(表1[[#This Row],[Credit_Score]]&lt;$J$12, "Decline", IF(表1[[#This Row],[Debt_to_Income]]&gt;=$J$13, "Review", "Approve"))</f>
+        <v>Approve</v>
+      </c>
       <c r="I3" t="s">
         <v>15</v>
       </c>
@@ -1693,6 +2829,10 @@
         <f>IF(表1[[#This Row],[Credit_Score]]&lt; $J$9, "High", "Low")</f>
         <v>Low</v>
       </c>
+      <c r="H4" t="str">
+        <f>IF(表1[[#This Row],[Credit_Score]]&lt;$J$12, "Decline", IF(表1[[#This Row],[Debt_to_Income]]&gt;=$J$13, "Review", "Approve"))</f>
+        <v>Approve</v>
+      </c>
       <c r="I4" t="s">
         <v>16</v>
       </c>
@@ -1725,6 +2865,10 @@
         <f>IF(表1[[#This Row],[Credit_Score]]&lt; $J$9, "High", "Low")</f>
         <v>High</v>
       </c>
+      <c r="H5" t="str">
+        <f>IF(表1[[#This Row],[Credit_Score]]&lt;$J$12, "Decline", IF(表1[[#This Row],[Debt_to_Income]]&gt;=$J$13, "Review", "Approve"))</f>
+        <v>Review</v>
+      </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -1750,6 +2894,10 @@
         <f>IF(表1[[#This Row],[Credit_Score]]&lt; $J$9, "High", "Low")</f>
         <v>High</v>
       </c>
+      <c r="H6" t="str">
+        <f>IF(表1[[#This Row],[Credit_Score]]&lt;$J$12, "Decline", IF(表1[[#This Row],[Debt_to_Income]]&gt;=$J$13, "Review", "Approve"))</f>
+        <v>Review</v>
+      </c>
       <c r="I6" t="s">
         <v>22</v>
       </c>
@@ -1781,6 +2929,10 @@
         <f>IF(表1[[#This Row],[Credit_Score]]&lt; $J$9, "High", "Low")</f>
         <v>High</v>
       </c>
+      <c r="H7" t="str">
+        <f>IF(表1[[#This Row],[Credit_Score]]&lt;$J$12, "Decline", IF(表1[[#This Row],[Debt_to_Income]]&gt;=$J$13, "Review", "Approve"))</f>
+        <v>Decline</v>
+      </c>
       <c r="I7" t="s">
         <v>19</v>
       </c>
@@ -1806,17 +2958,71 @@
         <v>3</v>
       </c>
     </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I12" t="s">
+        <v>24</v>
+      </c>
+      <c r="J12">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I13" t="s">
+        <v>25</v>
+      </c>
+      <c r="J13" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I15" t="s">
+        <v>26</v>
+      </c>
+      <c r="J15">
+        <f>COUNTIF(表1[Decision], "Approve")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="I16" t="s">
+        <v>27</v>
+      </c>
+      <c r="J16">
+        <f>COUNTIF(表1[Decision],"Review")</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="9:10" x14ac:dyDescent="0.3">
+      <c r="I17" t="s">
+        <v>28</v>
+      </c>
+      <c r="J17">
+        <f>COUNTIF(表1[Decision],"Decline")</f>
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="G2:G7">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Low">
+    <cfRule type="containsText" dxfId="10" priority="4" operator="containsText" text="Low">
       <formula>NOT(ISERROR(SEARCH("Low",G2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="High">
+    <cfRule type="containsText" dxfId="9" priority="5" operator="containsText" text="High">
       <formula>NOT(ISERROR(SEARCH("High",G2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="High">
+    <cfRule type="containsText" dxfId="8" priority="6" operator="containsText" text="High">
       <formula>NOT(ISERROR(SEARCH("High",G2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H7">
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="Approve">
+      <formula>NOT(ISERROR(SEARCH("Approve",H2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Review">
+      <formula>NOT(ISERROR(SEARCH("Review",H2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Decline">
+      <formula>NOT(ISERROR(SEARCH("Decline",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: add SQL applicant analysis script
</commit_message>
<xml_diff>
--- a/reports/excel/synthetic_credit_risk_prototype.xlsx
+++ b/reports/excel/synthetic_credit_risk_prototype.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5476D19E-1DB8-455B-A682-66E633D40C3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="15370" xr2:uid="{BBB7CC6D-377D-4AE4-9941-B0252BEF4F25}"/>
+    <workbookView xWindow="1550" yWindow="1520" windowWidth="23040" windowHeight="13400" xr2:uid="{BBB7CC6D-377D-4AE4-9941-B0252BEF4F25}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -220,10 +220,10 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="百分比" xfId="1" builtinId="5"/>
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="23">
+  <dxfs count="11">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -251,117 +251,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -423,7 +312,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="zh-CN"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -813,7 +702,7 @@
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="zh-CN"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -884,7 +773,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="zh-CN"/>
+          <a:endParaRPr lang="zh-CN" altLang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -2351,17 +2240,17 @@
   </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{5DB3054D-B453-4F4B-ABDE-676A06796AF5}" name="Applicant_ID"/>
-    <tableColumn id="2" xr3:uid="{C84C28F8-3796-47D7-9032-662F1557773A}" name="Income" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{9BFBAFA3-DE7A-4B0C-957A-D916E0E54EEB}" name="Debt" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{C84C28F8-3796-47D7-9032-662F1557773A}" name="Income" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{9BFBAFA3-DE7A-4B0C-957A-D916E0E54EEB}" name="Debt" dataDxfId="9"/>
     <tableColumn id="4" xr3:uid="{DC3D9AA5-71BF-43FA-9B0E-8A4F6512FB97}" name="Credit_Score"/>
     <tableColumn id="5" xr3:uid="{78414401-7D35-4508-9F47-09AEC9F83448}" name="Defaulted"/>
-    <tableColumn id="6" xr3:uid="{6C483C90-A97B-4157-8B4B-2DED3C5C25D4}" name="Debt_to_Income" dataDxfId="20" dataCellStyle="百分比">
+    <tableColumn id="6" xr3:uid="{6C483C90-A97B-4157-8B4B-2DED3C5C25D4}" name="Debt_to_Income" dataDxfId="8">
       <calculatedColumnFormula>表1[[#This Row],[Debt]]/表1[[#This Row],[Income]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{68BC03E3-32DD-4531-87E8-8A72C88C7D4F}" name="Risk_Flag" dataDxfId="19">
+    <tableColumn id="7" xr3:uid="{68BC03E3-32DD-4531-87E8-8A72C88C7D4F}" name="Risk_Flag" dataDxfId="7">
       <calculatedColumnFormula>IF(表1[[#This Row],[Credit_Score]]&lt; $J$9, "High", "Low")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{3075087F-CBFA-4972-B1FA-427EEF5F89D6}" name="Decision" dataDxfId="18">
+    <tableColumn id="8" xr3:uid="{3075087F-CBFA-4972-B1FA-427EEF5F89D6}" name="Decision" dataDxfId="6">
       <calculatedColumnFormula>IF(表1[[#This Row],[Credit_Score]]&lt;$J$12, "Decline", IF(表1[[#This Row],[Debt_to_Income]]&gt;=$J$13, "Review", "Approve"))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -2370,7 +2259,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -3004,25 +2893,25 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="G2:G7">
-    <cfRule type="containsText" dxfId="10" priority="4" operator="containsText" text="Low">
+    <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="Low">
       <formula>NOT(ISERROR(SEARCH("Low",G2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="9" priority="5" operator="containsText" text="High">
+    <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="High">
       <formula>NOT(ISERROR(SEARCH("High",G2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="6" operator="containsText" text="High">
+    <cfRule type="containsText" dxfId="3" priority="6" operator="containsText" text="High">
       <formula>NOT(ISERROR(SEARCH("High",G2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H2:H7">
-    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="Approve">
-      <formula>NOT(ISERROR(SEARCH("Approve",H2)))</formula>
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Decline">
+      <formula>NOT(ISERROR(SEARCH("Decline",H2)))</formula>
     </cfRule>
     <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Review">
       <formula>NOT(ISERROR(SEARCH("Review",H2)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Decline">
-      <formula>NOT(ISERROR(SEARCH("Decline",H2)))</formula>
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="Approve">
+      <formula>NOT(ISERROR(SEARCH("Approve",H2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>